<commit_message>
finished distress robot PCB and DC motor differential control code
</commit_message>
<xml_diff>
--- a/distress_call_robot/Mechanics/BOM.xlsx
+++ b/distress_call_robot/Mechanics/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -55,6 +55,9 @@
     <t xml:space="preserve">PCB</t>
   </si>
   <si>
+    <t xml:space="preserve">l7805</t>
+  </si>
+  <si>
     <t xml:space="preserve">Raspberry Pi Pico W</t>
   </si>
   <si>
@@ -80,9 +83,6 @@
   </si>
   <si>
     <t xml:space="preserve">MAX9814 Microphone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SPH0645 Microphone</t>
   </si>
   <si>
     <t xml:space="preserve">Batteries</t>
@@ -455,7 +455,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultColWidth="10.5234375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.53125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.95"/>
@@ -541,81 +541,80 @@
         <v>11</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>750</v>
+        <v>10</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="12" t="n">
         <f aca="false">C4*D4</f>
-        <v>750</v>
+        <v>10</v>
       </c>
       <c r="F4" s="13"/>
-      <c r="G4" s="12" t="s">
-        <v>12</v>
-      </c>
+      <c r="G4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>4.5</v>
+        <v>750</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="12" t="n">
         <f aca="false">C5*D5</f>
-        <v>9</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>14</v>
-      </c>
+        <v>750</v>
+      </c>
+      <c r="F5" s="13"/>
       <c r="G5" s="12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>30</v>
+        <v>4.5</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="12" t="n">
         <f aca="false">C6*D6</f>
-        <v>30</v>
+        <v>9</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>15</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="12" t="n">
         <f aca="false">C7*D7</f>
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="G7" s="12" t="s">
         <v>9</v>
@@ -623,83 +622,83 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">C8*D8</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">C9*D9</f>
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>175</v>
+        <v>2.5</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">C10*D10</f>
-        <v>350</v>
+        <v>7.5</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>480</v>
+        <v>175</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">C11*D11</f>
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>9</v>
@@ -745,7 +744,7 @@
         <v>23</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -841,7 +840,7 @@
       <c r="D20" s="20"/>
       <c r="E20" s="21" t="n">
         <f aca="false">SUM(E2:E19)</f>
-        <v>6561.5</v>
+        <v>6266.5</v>
       </c>
       <c r="F20" s="22"/>
       <c r="G20" s="23"/>

</xml_diff>

<commit_message>
finished GPS, distress call code and many more
</commit_message>
<xml_diff>
--- a/distress_call_robot/Mechanics/BOM.xlsx
+++ b/distress_call_robot/Mechanics/BOM.xlsx
@@ -168,12 +168,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFCCCCCC"/>
+        <bgColor rgb="FFCCCCFF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -261,6 +261,13 @@
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
       <top style="thin"/>
       <bottom style="thin"/>
       <diagonal/>
@@ -340,64 +347,48 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -409,31 +400,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -446,6 +449,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFCCCCCC"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -455,395 +518,405 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultColWidth="10.53125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="27.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="27.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.5"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="1" width="10.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="s">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="6" t="n">
+      <c r="C2" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="7" t="n">
+      <c r="D2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="8" t="n">
         <f aca="false">C2*D2</f>
         <v>45</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="11" t="n">
+      <c r="C3" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="D3" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="12" t="n">
+      <c r="D3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13" t="n">
         <f aca="false">C3*D3</f>
         <v>80</v>
       </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="12"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="D4" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="12" t="n">
+      <c r="D4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="13" t="n">
         <f aca="false">C4*D4</f>
         <v>10</v>
       </c>
-      <c r="F4" s="13"/>
-      <c r="G4" s="12"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="12" t="n">
         <v>750</v>
       </c>
-      <c r="D5" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="12" t="n">
+      <c r="D5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="13" t="n">
         <f aca="false">C5*D5</f>
         <v>750</v>
       </c>
-      <c r="F5" s="13"/>
-      <c r="G5" s="12" t="s">
+      <c r="F5" s="14"/>
+      <c r="G5" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="12" t="n">
         <v>4.5</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="13" t="n">
         <f aca="false">C6*D6</f>
         <v>9</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="D7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="12" t="n">
+      <c r="D7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="13" t="n">
         <f aca="false">C7*D7</f>
         <v>30</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="F7" s="15"/>
+      <c r="G7" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="12" t="n">
+      <c r="D8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="13" t="n">
         <f aca="false">C8*D8</f>
         <v>2</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="F8" s="15"/>
+      <c r="G8" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="11" t="n">
+      <c r="C9" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="13" t="n">
         <f aca="false">C9*D9</f>
         <v>3</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="F9" s="15"/>
+      <c r="G9" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="12" t="n">
         <v>2.5</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="13" t="n">
         <f aca="false">C10*D10</f>
         <v>7.5</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="F10" s="15"/>
+      <c r="G10" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="12" t="n">
         <v>175</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">C11*D11</f>
         <v>525</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="F11" s="15"/>
+      <c r="G11" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">C12*D12</f>
         <v>0</v>
       </c>
-      <c r="G12" s="12"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>85</v>
       </c>
-      <c r="D13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="12" t="n">
+      <c r="D13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="13" t="n">
         <f aca="false">C13*D13</f>
         <v>85</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="G13" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="12" t="n">
         <v>580</v>
       </c>
-      <c r="D14" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="12" t="n">
+      <c r="D14" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="13" t="n">
         <f aca="false">C14*D14</f>
         <v>580</v>
       </c>
-      <c r="G14" s="12"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="13"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="10" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="12" t="n">
         <v>70</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="13" t="n">
         <f aca="false">C16*D16</f>
         <v>140</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="F16" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="12"/>
+      <c r="G16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="12"/>
-      <c r="G17" s="12"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14"/>
-      <c r="B18" s="15" t="s">
+      <c r="A18" s="5"/>
+      <c r="B18" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="16" t="n">
+      <c r="C18" s="12" t="n">
         <v>4000</v>
       </c>
-      <c r="D18" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="16" t="n">
+      <c r="D18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="12" t="n">
         <f aca="false">C18*D18</f>
         <v>4000</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="G18" s="12"/>
+      <c r="G18" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="12"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="13"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1"/>
-      <c r="B20" s="19" t="s">
+      <c r="A20" s="2"/>
+      <c r="B20" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="21" t="n">
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="20" t="n">
         <f aca="false">SUM(E2:E19)</f>
         <v>6266.5</v>
       </c>
-      <c r="F20" s="22"/>
-      <c r="G20" s="23"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="22"/>
     </row>
     <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>